<commit_message>
update dashboard and excel workbooks
</commit_message>
<xml_diff>
--- a/Dashboard_LaaS_vs_NYTG/new_models/通用版_能源托管_vs_LaaS_财务模型_v3_逻辑复核版__FILLED_01_Tier01_UniformAI_80_WPS.xlsx
+++ b/Dashboard_LaaS_vs_NYTG/new_models/通用版_能源托管_vs_LaaS_财务模型_v3_逻辑复核版__FILLED_01_Tier01_UniformAI_80_WPS.xlsx
@@ -1055,7 +1055,7 @@
       </s:c>
       <s:c r="C6" s="168">
         <s:f>'03_Baseline'!D5</s:f>
-        <s:v/>
+        <s:v>4568.0</s:v>
       </s:c>
       <s:c r="D6" s="130" t="inlineStr">
         <s:is>
@@ -1081,7 +1081,7 @@
       </s:c>
       <s:c r="C7" s="169">
         <s:f>'03_Baseline'!D11</s:f>
-        <s:v/>
+        <s:v>0.6900001496778997</s:v>
       </s:c>
       <s:c r="D7" s="130" t="inlineStr">
         <s:is>
@@ -1107,7 +1107,7 @@
       </s:c>
       <s:c r="C8" s="170">
         <s:f>'03_Baseline'!D12</s:f>
-        <s:v/>
+        <s:v>2120554.0</s:v>
       </s:c>
       <s:c r="D8" s="130" t="inlineStr">
         <s:is>
@@ -1133,7 +1133,7 @@
       </s:c>
       <s:c r="C9" s="170">
         <s:f>'03_Baseline'!D14</s:f>
-        <s:v/>
+        <s:v>609997.0</s:v>
       </s:c>
       <s:c r="D9" s="130" t="inlineStr">
         <s:is>
@@ -1159,7 +1159,7 @@
       </s:c>
       <s:c r="C10" s="170">
         <s:f>'03_Baseline'!D16</s:f>
-        <s:v/>
+        <s:v>2600000.0</s:v>
       </s:c>
       <s:c r="D10" s="130" t="inlineStr">
         <s:is>
@@ -1185,7 +1185,7 @@
       </s:c>
       <s:c r="C11" s="130">
         <s:f>'04_Mode_Params'!C6='04_Mode_Params'!D6</s:f>
-        <s:v/>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="D11" s="130" t="inlineStr">
         <s:is>
@@ -1269,7 +1269,7 @@
       </s:c>
       <s:c r="C15" s="171">
         <s:f>'04_Mode_Params'!C8</s:f>
-        <s:v>0.5</s:v>
+        <s:v>0.515219607706288</s:v>
       </s:c>
       <s:c r="D15" s="171">
         <s:f>'04_Mode_Params'!D8</s:f>
@@ -1308,11 +1308,11 @@
       </s:c>
       <s:c r="C16" s="172">
         <s:f>'03_Baseline'!D10*'04_Mode_Params'!C8</s:f>
-        <s:v>2056000.0</s:v>
+        <s:v>1583406.902897073</s:v>
       </s:c>
       <s:c r="D16" s="172">
         <s:f>'03_Baseline'!D10*'04_Mode_Params'!D8</s:f>
-        <s:v>3289600.0</s:v>
+        <s:v>2458612.8000000003</s:v>
       </s:c>
       <s:c r="E16" s="172">
         <s:f>D16-C16</s:f>
@@ -1347,11 +1347,11 @@
       </s:c>
       <s:c r="C17" s="172">
         <s:f>'03_Baseline'!D12-'04_Mode_Params'!C9</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1092551.0</s:v>
       </s:c>
       <s:c r="D17" s="172">
         <s:f>'03_Baseline'!D12-'04_Mode_Params'!D9</s:f>
-        <s:v>1644800.0</s:v>
+        <s:v>1696443.2000000002</s:v>
       </s:c>
       <s:c r="E17" s="172">
         <s:f>D17-C17</s:f>
@@ -1386,15 +1386,15 @@
       </s:c>
       <s:c r="C18" s="173">
         <s:f>'04_Mode_Params'!C19</s:f>
-        <s:v/>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="D18" s="173">
         <s:f>'04_Mode_Params'!D19</s:f>
-        <s:v/>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="E18" s="173">
         <s:f>C18-D18</s:f>
-        <s:v/>
+        <s:v>646192.2000000002</s:v>
       </s:c>
       <s:c r="F18" s="45" t="inlineStr">
         <s:is>
@@ -1425,15 +1425,15 @@
       </s:c>
       <s:c r="C19" s="173">
         <s:f>'04_Mode_Params'!C20</s:f>
-        <s:v/>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="D19" s="173">
         <s:f>'04_Mode_Params'!D20</s:f>
-        <s:v/>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="E19" s="173">
         <s:f>D19-C19</s:f>
-        <s:v/>
+        <s:v>646192.2000000002</s:v>
       </s:c>
       <s:c r="F19" s="45" t="inlineStr">
         <s:is>
@@ -1464,15 +1464,15 @@
       </s:c>
       <s:c r="C20" s="173">
         <s:f>'04_Mode_Params'!C16</s:f>
-        <s:v/>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="D20" s="173">
         <s:f>'04_Mode_Params'!D16</s:f>
-        <s:v/>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="E20" s="173">
         <s:f>D20-C20</s:f>
-        <s:v/>
+        <s:v>-42300.0</s:v>
       </s:c>
       <s:c r="F20" s="45" t="inlineStr">
         <s:is>
@@ -1503,15 +1503,15 @@
       </s:c>
       <s:c r="C21" s="173">
         <s:f>'04_Mode_Params'!C17</s:f>
-        <s:v/>
+        <s:v>609997.0</s:v>
       </s:c>
       <s:c r="D21" s="173">
         <s:f>'04_Mode_Params'!D17</s:f>
-        <s:v/>
+        <s:v>327599.9999999999</s:v>
       </s:c>
       <s:c r="E21" s="173">
         <s:f>C21-D21</s:f>
-        <s:v/>
+        <s:v>282397.0000000001</s:v>
       </s:c>
       <s:c r="F21" s="45" t="inlineStr">
         <s:is>
@@ -1542,15 +1542,15 @@
       </s:c>
       <s:c r="C22" s="173">
         <s:f>'04_Mode_Params'!C13</s:f>
-        <s:v/>
+        <s:v>394236.8839841539</s:v>
       </s:c>
       <s:c r="D22" s="173">
         <s:f>'04_Mode_Params'!D13</s:f>
-        <s:v/>
+        <s:v>115993.96444811902</s:v>
       </s:c>
       <s:c r="E22" s="173">
         <s:f>C22-D22</s:f>
-        <s:v/>
+        <s:v>278242.9195360349</s:v>
       </s:c>
       <s:c r="F22" s="45" t="inlineStr">
         <s:is>
@@ -1581,15 +1581,15 @@
       </s:c>
       <s:c r="C23" s="173">
         <s:f>'04_Mode_Params'!C14+'04_Mode_Params'!C15</s:f>
-        <s:v/>
+        <s:v>161820.08701188455</s:v>
       </s:c>
       <s:c r="D23" s="173">
         <s:f>'04_Mode_Params'!D14+'04_Mode_Params'!D15</s:f>
-        <s:v/>
+        <s:v>148124.2248863166</s:v>
       </s:c>
       <s:c r="E23" s="173">
         <s:f>C23-D23</s:f>
-        <s:v/>
+        <s:v>13695.862125567946</s:v>
       </s:c>
       <s:c r="F23" s="45" t="inlineStr">
         <s:is>
@@ -1620,15 +1620,15 @@
       </s:c>
       <s:c r="C24" s="173">
         <s:f>'04_Mode_Params'!C18</s:f>
-        <s:v/>
+        <s:v>1732303.0</s:v>
       </s:c>
       <s:c r="D24" s="173">
         <s:f>'04_Mode_Params'!D18</s:f>
-        <s:v/>
+        <s:v>1972400.0</s:v>
       </s:c>
       <s:c r="E24" s="173">
         <s:f>D24-C24</s:f>
-        <s:v/>
+        <s:v>240097.0</s:v>
       </s:c>
       <s:c r="F24" s="45" t="inlineStr">
         <s:is>
@@ -1659,15 +1659,15 @@
       </s:c>
       <s:c r="C25" s="173">
         <s:f>'04_Mode_Params'!C5</s:f>
-        <s:v/>
+        <s:v>3539400.0</s:v>
       </s:c>
       <s:c r="D25" s="173">
         <s:f>'04_Mode_Params'!D5</s:f>
-        <s:v/>
+        <s:v>3539400.0</s:v>
       </s:c>
       <s:c r="E25" s="173">
         <s:f>C25-D25</s:f>
-        <s:v/>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="F25" s="45" t="inlineStr">
         <s:is>
@@ -1698,15 +1698,15 @@
       </s:c>
       <s:c r="C26" s="173">
         <s:f>'05_Annual_Model'!M24</s:f>
-        <s:v/>
+        <s:v>13783630.0</s:v>
       </s:c>
       <s:c r="D26" s="173">
         <s:f>'05_Annual_Model'!M51</s:f>
-        <s:v/>
+        <s:v>16184599.999999976</s:v>
       </s:c>
       <s:c r="E26" s="173">
         <s:f>D26-C26</s:f>
-        <s:v/>
+        <s:v>2400969.999999976</s:v>
       </s:c>
       <s:c r="F26" s="45" t="inlineStr">
         <s:is>
@@ -1737,15 +1737,15 @@
       </s:c>
       <s:c r="C27" s="173">
         <s:f>'05_Annual_Model'!C25</s:f>
-        <s:v/>
+        <s:v>7423046.099119451</s:v>
       </s:c>
       <s:c r="D27" s="173">
         <s:f>'05_Annual_Model'!C52</s:f>
-        <s:v/>
+        <s:v>8205507.890886906</s:v>
       </s:c>
       <s:c r="E27" s="173">
         <s:f>D27-C27</s:f>
-        <s:v/>
+        <s:v>782461.7917674547</s:v>
       </s:c>
       <s:c r="F27" s="45" t="inlineStr">
         <s:is>
@@ -1776,15 +1776,15 @@
       </s:c>
       <s:c r="C28" s="171">
         <s:f>'05_Annual_Model'!C26</s:f>
-        <s:v/>
+        <s:v>0.4797080973744201</s:v>
       </s:c>
       <s:c r="D28" s="171">
         <s:f>'05_Annual_Model'!C53</s:f>
-        <s:v/>
+        <s:v>0.7200751553415916</s:v>
       </s:c>
       <s:c r="E28" s="171">
         <s:f>D28-C28</s:f>
-        <s:v/>
+        <s:v>0.2403670579671715</s:v>
       </s:c>
       <s:c r="F28" s="45" t="inlineStr">
         <s:is>
@@ -2674,11 +2674,11 @@
       </s:c>
       <s:c r="C18" s="173">
         <s:f>'05_Annual_Model'!M24</s:f>
-        <s:v>6730600.0</s:v>
+        <s:v>13783630.0</s:v>
       </s:c>
       <s:c r="D18" s="173">
         <s:f>'05_Annual_Model'!M51</s:f>
-        <s:v>15684600.0</s:v>
+        <s:v>16184599.999999976</s:v>
       </s:c>
       <s:c r="E18" s="173">
         <s:f>D18-C18</s:f>
@@ -2707,11 +2707,11 @@
       </s:c>
       <s:c r="C19" s="173">
         <s:f>'05_Annual_Model'!C25</s:f>
-        <s:v>2959712.5361993117</s:v>
+        <s:v>7423046.099119451</s:v>
       </s:c>
       <s:c r="D19" s="173">
         <s:f>'05_Annual_Model'!C52</s:f>
-        <s:v>7907776.500426378</s:v>
+        <s:v>8205507.890886906</s:v>
       </s:c>
       <s:c r="E19" s="173">
         <s:f>D19-C19</s:f>
@@ -2740,11 +2740,11 @@
       </s:c>
       <s:c r="C20" s="176">
         <s:f>'05_Annual_Model'!C26</s:f>
-        <s:v>0.2618003333030041</s:v>
+        <s:v>0.4797080973744201</s:v>
       </s:c>
       <s:c r="D20" s="176">
         <s:f>'05_Annual_Model'!C53</s:f>
-        <s:v>0.6965192371624709</s:v>
+        <s:v>0.7200751553415916</s:v>
       </s:c>
       <s:c r="E20" s="173">
         <s:f>D20-C20</s:f>
@@ -2773,11 +2773,11 @@
       </s:c>
       <s:c r="C21" s="171">
         <s:f>'05_Annual_Model'!C27</s:f>
-        <s:v>2.901621743798384</s:v>
+        <s:v>4.8943408487314235</s:v>
       </s:c>
       <s:c r="D21" s="171">
         <s:f>'05_Annual_Model'!C54</s:f>
-        <s:v>5.431429055772165</s:v>
+        <s:v>5.572695937164491</s:v>
       </s:c>
       <s:c r="E21" s="171">
         <s:f>D21-C21</s:f>
@@ -3234,7 +3234,7 @@
         </s:is>
       </s:c>
       <s:c r="D6" s="178" t="n">
-        <s:v>5000</s:v>
+        <s:v>4568</s:v>
       </s:c>
       <s:c r="E6" s="45" t="inlineStr">
         <s:is>
@@ -3274,7 +3274,7 @@
         </s:is>
       </s:c>
       <s:c r="D7" s="179" t="n">
-        <s:v>2342300</s:v>
+        <s:v>2600000</s:v>
       </s:c>
       <s:c r="E7" s="45" t="inlineStr">
         <s:is>
@@ -3314,7 +3314,7 @@
         </s:is>
       </s:c>
       <s:c r="D8" s="179" t="n">
-        <s:v>0.5</s:v>
+        <s:v>0.6900001496778997</s:v>
       </s:c>
       <s:c r="E8" s="45" t="inlineStr">
         <s:is>
@@ -3354,7 +3354,7 @@
         </s:is>
       </s:c>
       <s:c r="D9" s="180" t="n">
-        <s:v>204.8318804483188</s:v>
+        <s:v>167.5670046432707</s:v>
       </s:c>
       <s:c r="E9" s="45" t="inlineStr">
         <s:is>
@@ -3474,7 +3474,7 @@
         </s:is>
       </s:c>
       <s:c r="D12" s="178" t="n">
-        <s:v>122</s:v>
+        <s:v>133.536996497373</s:v>
       </s:c>
       <s:c r="E12" s="45" t="inlineStr">
         <s:is>
@@ -3714,7 +3714,7 @@
         </s:is>
       </s:c>
       <s:c r="D18" s="182" t="n">
-        <s:v>707.88</s:v>
+        <s:v>774.8248686514886</s:v>
       </s:c>
       <s:c r="E18" s="50" t="inlineStr">
         <s:is>
@@ -3754,7 +3754,7 @@
         </s:is>
       </s:c>
       <s:c r="D19" s="179" t="n">
-        <s:v>1637000</s:v>
+        <s:v>2342300</s:v>
       </s:c>
       <s:c r="E19" s="45" t="inlineStr">
         <s:is>
@@ -3834,7 +3834,7 @@
         </s:is>
       </s:c>
       <s:c r="D21" s="181" t="n">
-        <s:v>0.5</s:v>
+        <s:v>0.5152196077062881</s:v>
       </s:c>
       <s:c r="E21" s="45" t="inlineStr">
         <s:is>
@@ -3874,7 +3874,7 @@
         </s:is>
       </s:c>
       <s:c r="D22" s="179" t="n">
-        <s:v>81.33333333333333</s:v>
+        <s:v>86.30404640633843</s:v>
       </s:c>
       <s:c r="E22" s="45" t="inlineStr">
         <s:is>
@@ -3914,7 +3914,7 @@
         </s:is>
       </s:c>
       <s:c r="D23" s="179" t="n">
-        <s:v>152500</s:v>
+        <s:v>161820.0870118845</s:v>
       </s:c>
       <s:c r="E23" s="45" t="inlineStr">
         <s:is>
@@ -3954,7 +3954,7 @@
         </s:is>
       </s:c>
       <s:c r="D24" s="179" t="n">
-        <s:v>50833.33333333333</s:v>
+        <s:v>53940.02900396152</s:v>
       </s:c>
       <s:c r="E24" s="45" t="inlineStr">
         <s:is>
@@ -3994,7 +3994,7 @@
         </s:is>
       </s:c>
       <s:c r="D25" s="178" t="n">
-        <s:v>0</s:v>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="E25" s="45" t="inlineStr">
         <s:is>
@@ -4115,7 +4115,7 @@
       </s:c>
       <s:c r="D28" s="182">
         <s:f>VLOOKUP($D$48,$A$52:$G$54,3,FALSE)</s:f>
-        <s:v>707.88</s:v>
+        <s:v>774.8248686514886</s:v>
       </s:c>
       <s:c r="E28" s="50" t="inlineStr">
         <s:is>
@@ -4155,7 +4155,7 @@
         </s:is>
       </s:c>
       <s:c r="D29" s="179" t="n">
-        <s:v>2250000</s:v>
+        <s:v>2300000</s:v>
       </s:c>
       <s:c r="E29" s="45" t="inlineStr">
         <s:is>
@@ -4277,7 +4277,7 @@
       </s:c>
       <s:c r="D32" s="179">
         <s:f>VLOOKUP($D$48,$A$52:$G$54,4,FALSE)</s:f>
-        <s:v>24.56999999999999</s:v>
+        <s:v>25.392724266225706</s:v>
       </s:c>
       <s:c r="E32" s="45" t="inlineStr">
         <s:is>
@@ -4318,7 +4318,7 @@
       </s:c>
       <s:c r="D33" s="179">
         <s:f>VLOOKUP($D$48,$A$52:$G$54,5,FALSE)</s:f>
-        <s:v>143324.99999999994</s:v>
+        <s:v>148124.2248863166</s:v>
       </s:c>
       <s:c r="E33" s="45" t="inlineStr">
         <s:is>
@@ -4359,7 +4359,7 @@
       </s:c>
       <s:c r="D34" s="179">
         <s:f>VLOOKUP($D$48,$A$52:$G$54,6,FALSE)</s:f>
-        <s:v>61424.99999999998</s:v>
+        <s:v>63481.81066556426</s:v>
       </s:c>
       <s:c r="E34" s="45" t="inlineStr">
         <s:is>
@@ -4399,7 +4399,7 @@
         </s:is>
       </s:c>
       <s:c r="D35" s="178" t="n">
-        <s:v>0</s:v>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="E35" s="45" t="inlineStr">
         <s:is>
@@ -4559,6 +4559,16 @@
         </s:is>
       </s:c>
     </s:row>
+    <s:row r="49">
+      <s:c r="A49" t="inlineStr">
+        <s:is>
+          <s:t>灯杆数量(根)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D49" t="n">
+        <s:v>2345</s:v>
+      </s:c>
+    </s:row>
     <s:row r="50">
       <s:c r="A50" s="183" t="inlineStr">
         <s:is>
@@ -4619,16 +4629,16 @@
         <s:v>0.5869565217391304</s:v>
       </s:c>
       <s:c r="C52" s="186" t="n">
-        <s:v>707.88</s:v>
+        <s:v>774.8248686514886</s:v>
       </s:c>
       <s:c r="D52" s="186" t="n">
-        <s:v>24.56999999999999</s:v>
+        <s:v>25.39272426622571</s:v>
       </s:c>
       <s:c r="E52" s="186" t="n">
-        <s:v>143324.9999999999</s:v>
+        <s:v>148124.2248863166</s:v>
       </s:c>
       <s:c r="F52" s="186" t="n">
-        <s:v>61424.99999999998</s:v>
+        <s:v>63481.81066556426</s:v>
       </s:c>
       <s:c r="G52" s="185" t="inlineStr">
         <s:is>
@@ -4646,16 +4656,16 @@
         <s:v>0.6458333333333333</s:v>
       </s:c>
       <s:c r="C53" s="186" t="n">
-        <s:v>775.9100259740259</s:v>
+        <s:v>849.2885573270861</s:v>
       </s:c>
       <s:c r="D53" s="186" t="n">
-        <s:v>23.80749999999999</s:v>
+        <s:v>24.60469202149648</s:v>
       </s:c>
       <s:c r="E53" s="186" t="n">
-        <s:v>138877.0833333333</s:v>
+        <s:v>143527.3701253961</s:v>
       </s:c>
       <s:c r="F53" s="186" t="n">
-        <s:v>59518.74999999999</s:v>
+        <s:v>61511.7300537412</s:v>
       </s:c>
       <s:c r="G53" s="185" t="inlineStr">
         <s:is>
@@ -4673,16 +4683,16 @@
         <s:v>0.999</s:v>
       </s:c>
       <s:c r="C54" s="186" t="n">
-        <s:v>671.1070129870129</s:v>
+        <s:v>734.5742261241385</s:v>
       </s:c>
       <s:c r="D54" s="186" t="n">
-        <s:v>7.624999999999998</s:v>
+        <s:v>7.880322447292269</s:v>
       </s:c>
       <s:c r="E54" s="186" t="n">
-        <s:v>44479.16666666666</s:v>
+        <s:v>45968.54760920489</s:v>
       </s:c>
       <s:c r="F54" s="186" t="n">
-        <s:v>19062.5</s:v>
+        <s:v>19700.80611823067</s:v>
       </s:c>
       <s:c r="G54" s="185" t="inlineStr">
         <s:is>
@@ -4707,427 +4717,435 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Z18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>现状基准测算｜不改造情形</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="18" t="n"/>
-      <c r="H1" s="18" t="n"/>
-      <c r="I1" s="18" t="n"/>
-      <c r="J1" s="18" t="n"/>
-      <c r="K1" s="18" t="n"/>
-      <c r="L1" s="18" t="n"/>
-      <c r="M1" s="18" t="n"/>
-      <c r="N1" s="18" t="n"/>
-      <c r="O1" s="18" t="n"/>
-      <c r="P1" s="18" t="n"/>
-      <c r="Q1" s="18" t="n"/>
-      <c r="R1" s="18" t="n"/>
-      <c r="S1" s="18" t="n"/>
-      <c r="T1" s="18" t="n"/>
-      <c r="U1" s="18" t="n"/>
-      <c r="V1" s="18" t="n"/>
-      <c r="W1" s="18" t="n"/>
-      <c r="X1" s="18" t="n"/>
-      <c r="Y1" s="18" t="n"/>
-      <c r="Z1" s="18" t="n"/>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>所有节省额均相对于本页“不改造”基准计算。</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n"/>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="44" t="inlineStr">
-        <is>
-          <t>项目</t>
-        </is>
-      </c>
-      <c r="B4" s="44" t="inlineStr">
-        <is>
-          <t>单位</t>
-        </is>
-      </c>
-      <c r="C4" s="44" t="inlineStr">
-        <is>
-          <t>公式/口径</t>
-        </is>
-      </c>
-      <c r="D4" s="44" t="inlineStr">
-        <is>
-          <t>计算值</t>
-        </is>
-      </c>
-      <c r="E4" s="44" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
-      <c r="F4" s="44" t="inlineStr">
-        <is>
-          <t>校验</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="45" t="inlineStr">
-        <is>
-          <t>灯具数量</t>
-        </is>
-      </c>
-      <c r="B5" s="45" t="inlineStr">
-        <is>
-          <t>盏</t>
-        </is>
-      </c>
-      <c r="C5" s="60" t="inlineStr">
-        <is>
-          <t>来自Inputs</t>
-        </is>
-      </c>
-      <c r="D5" s="187">
-        <f>'02_Inputs'!D6</f>
-        <v/>
-      </c>
-      <c r="E5" s="60" t="str"/>
-      <c r="F5" s="45" t="str"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="45" t="inlineStr">
-        <is>
-          <t>现状单灯功率</t>
-        </is>
-      </c>
-      <c r="B6" s="45" t="inlineStr">
-        <is>
-          <t>W/盏</t>
-        </is>
-      </c>
-      <c r="C6" s="60" t="inlineStr">
-        <is>
-          <t>来自Inputs</t>
-        </is>
-      </c>
-      <c r="D6" s="187">
-        <f>'02_Inputs'!D9</f>
-        <v/>
-      </c>
-      <c r="E6" s="60" t="str"/>
-      <c r="F6" s="45" t="str"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="45" t="inlineStr">
-        <is>
-          <t>每日亮灯小时</t>
-        </is>
-      </c>
-      <c r="B7" s="45" t="inlineStr">
-        <is>
-          <t>小时/天</t>
-        </is>
-      </c>
-      <c r="C7" s="60" t="inlineStr">
-        <is>
-          <t>来自Inputs</t>
-        </is>
-      </c>
-      <c r="D7" s="187">
-        <f>'02_Inputs'!D10</f>
-        <v/>
-      </c>
-      <c r="E7" s="60" t="str"/>
-      <c r="F7" s="45" t="str"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="45" t="inlineStr">
-        <is>
-          <t>年运行天数</t>
-        </is>
-      </c>
-      <c r="B8" s="45" t="inlineStr">
-        <is>
-          <t>天/年</t>
-        </is>
-      </c>
-      <c r="C8" s="60" t="inlineStr">
-        <is>
-          <t>来自Inputs</t>
-        </is>
-      </c>
-      <c r="D8" s="187">
-        <f>'02_Inputs'!D11</f>
-        <v/>
-      </c>
-      <c r="E8" s="60" t="str"/>
-      <c r="F8" s="45" t="str"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="45" t="inlineStr">
-        <is>
-          <t>年运行小时</t>
-        </is>
-      </c>
-      <c r="B9" s="45" t="inlineStr">
-        <is>
-          <t>小时/年</t>
-        </is>
-      </c>
-      <c r="C9" s="60" t="inlineStr">
-        <is>
-          <t>每日亮灯小时×年运行天数</t>
-        </is>
-      </c>
-      <c r="D9" s="187">
-        <f>D7*D8</f>
-        <v/>
-      </c>
-      <c r="E9" s="60" t="str"/>
-      <c r="F9" s="45" t="str"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="45" t="inlineStr">
-        <is>
-          <t>现状年用电量</t>
-        </is>
-      </c>
-      <c r="B10" s="45" t="inlineStr">
-        <is>
-          <t>kWh/年</t>
-        </is>
-      </c>
-      <c r="C10" s="60" t="inlineStr">
-        <is>
-          <t>灯具数量×单灯功率÷1000×年运行小时</t>
-        </is>
-      </c>
-      <c r="D10" s="187">
-        <f>D5*D6/1000*D9</f>
-        <v/>
-      </c>
-      <c r="E10" s="60" t="str"/>
-      <c r="F10" s="45" t="str"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="45" t="inlineStr">
-        <is>
-          <t>电价</t>
-        </is>
-      </c>
-      <c r="B11" s="45" t="inlineStr">
-        <is>
-          <t>元/kWh</t>
-        </is>
-      </c>
-      <c r="C11" s="60" t="inlineStr">
-        <is>
-          <t>来自Inputs</t>
-        </is>
-      </c>
-      <c r="D11" s="188">
-        <f>'02_Inputs'!D8</f>
-        <v/>
-      </c>
-      <c r="E11" s="60" t="str"/>
-      <c r="F11" s="45" t="str"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="45" t="inlineStr">
-        <is>
-          <t>基准年电费</t>
-        </is>
-      </c>
-      <c r="B12" s="45" t="inlineStr">
-        <is>
-          <t>元/年</t>
-        </is>
-      </c>
-      <c r="C12" s="60" t="inlineStr">
-        <is>
-          <t>现状年用电量×电价</t>
-        </is>
-      </c>
-      <c r="D12" s="189">
-        <f>D10*D11</f>
-        <v/>
-      </c>
-      <c r="E12" s="60" t="str"/>
-      <c r="F12" s="45" t="str"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="45" t="inlineStr">
-        <is>
-          <t>现状运维单价</t>
-        </is>
-      </c>
-      <c r="B13" s="45" t="inlineStr">
-        <is>
-          <t>元/盏/年</t>
-        </is>
-      </c>
-      <c r="C13" s="60" t="inlineStr">
-        <is>
-          <t>来自Inputs</t>
-        </is>
-      </c>
-      <c r="D13" s="189">
-        <f>'02_Inputs'!D12</f>
-        <v/>
-      </c>
-      <c r="E13" s="60" t="str"/>
-      <c r="F13" s="45" t="str"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="45" t="inlineStr">
-        <is>
-          <t>基准年运维费</t>
-        </is>
-      </c>
-      <c r="B14" s="45" t="inlineStr">
-        <is>
-          <t>元/年</t>
-        </is>
-      </c>
-      <c r="C14" s="60" t="inlineStr">
-        <is>
-          <t>灯具数量×现状运维单价</t>
-        </is>
-      </c>
-      <c r="D14" s="189">
-        <f>D5*D13</f>
-        <v/>
-      </c>
-      <c r="E14" s="60" t="str"/>
-      <c r="F14" s="45" t="str"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="79" t="inlineStr">
-        <is>
-          <t>基准年总成本</t>
-        </is>
-      </c>
-      <c r="B15" s="79" t="inlineStr">
-        <is>
-          <t>元/年</t>
-        </is>
-      </c>
-      <c r="C15" s="89" t="inlineStr">
-        <is>
-          <t>基准年电费+基准年运维费</t>
-        </is>
-      </c>
-      <c r="D15" s="190">
-        <f>D12+D14</f>
-        <v/>
-      </c>
-      <c r="E15" s="89" t="str"/>
-      <c r="F15" s="79" t="str"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="79" t="inlineStr">
-        <is>
-          <t>业主年度服务费预算</t>
-        </is>
-      </c>
-      <c r="B16" s="79" t="inlineStr">
-        <is>
-          <t>元/年</t>
-        </is>
-      </c>
-      <c r="C16" s="89" t="inlineStr">
-        <is>
-          <t>来自Inputs</t>
-        </is>
-      </c>
-      <c r="D16" s="190">
-        <f>'02_Inputs'!D7</f>
-        <v/>
-      </c>
-      <c r="E16" s="89" t="str"/>
-      <c r="F16" s="79" t="str"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="79" t="inlineStr">
-        <is>
-          <t>10年业主预算总额</t>
-        </is>
-      </c>
-      <c r="B17" s="79" t="inlineStr">
-        <is>
-          <t>元</t>
-        </is>
-      </c>
-      <c r="C17" s="89" t="inlineStr">
-        <is>
-          <t>年度预算×模型期</t>
-        </is>
-      </c>
-      <c r="D17" s="190">
-        <f>D16*'02_Inputs'!D5</f>
-        <v/>
-      </c>
-      <c r="E17" s="89" t="str"/>
-      <c r="F17" s="79" t="str"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="79" t="inlineStr">
-        <is>
-          <t>10年不改造总成本</t>
-        </is>
-      </c>
-      <c r="B18" s="79" t="inlineStr">
-        <is>
-          <t>元</t>
-        </is>
-      </c>
-      <c r="C18" s="89" t="inlineStr">
-        <is>
-          <t>年度基准总成本合计，考虑增长率</t>
-        </is>
-      </c>
-      <c r="D18" s="190">
-        <f>SUM('05_Annual_Model'!D8:M8)</f>
-        <v/>
-      </c>
-      <c r="E18" s="89" t="str"/>
-      <c r="F18" s="79" t="str"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<s:worksheet xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <s:sheetPr>
+    <s:outlinePr summaryBelow="1" summaryRight="1"/>
+    <s:pageSetUpPr/>
+  </s:sheetPr>
+  <s:dimension ref="A1:Z18"/>
+  <s:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <s:cols>
+    <s:col width="24" customWidth="1" min="1" max="1"/>
+    <s:col width="14" customWidth="1" min="2" max="2"/>
+    <s:col width="46" customWidth="1" min="3" max="3"/>
+    <s:col width="18" customWidth="1" min="4" max="4"/>
+    <s:col width="34" customWidth="1" min="5" max="5"/>
+    <s:col width="16" customWidth="1" min="6" max="6"/>
+  </s:cols>
+  <s:sheetData>
+    <s:row r="1" ht="26" customHeight="1">
+      <s:c r="A1" s="5" t="inlineStr">
+        <s:is>
+          <s:t>现状基准测算｜不改造情形</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B1" s="1" t="n"/>
+      <s:c r="C1" s="1" t="n"/>
+      <s:c r="D1" s="1" t="n"/>
+      <s:c r="E1" s="1" t="n"/>
+      <s:c r="F1" s="1" t="n"/>
+      <s:c r="G1" s="18" t="n"/>
+      <s:c r="H1" s="18" t="n"/>
+      <s:c r="I1" s="18" t="n"/>
+      <s:c r="J1" s="18" t="n"/>
+      <s:c r="K1" s="18" t="n"/>
+      <s:c r="L1" s="18" t="n"/>
+      <s:c r="M1" s="18" t="n"/>
+      <s:c r="N1" s="18" t="n"/>
+      <s:c r="O1" s="18" t="n"/>
+      <s:c r="P1" s="18" t="n"/>
+      <s:c r="Q1" s="18" t="n"/>
+      <s:c r="R1" s="18" t="n"/>
+      <s:c r="S1" s="18" t="n"/>
+      <s:c r="T1" s="18" t="n"/>
+      <s:c r="U1" s="18" t="n"/>
+      <s:c r="V1" s="18" t="n"/>
+      <s:c r="W1" s="18" t="n"/>
+      <s:c r="X1" s="18" t="n"/>
+      <s:c r="Y1" s="18" t="n"/>
+      <s:c r="Z1" s="18" t="n"/>
+    </s:row>
+    <s:row r="2" ht="22" customHeight="1">
+      <s:c r="A2" s="7" t="inlineStr">
+        <s:is>
+          <s:t>所有节省额均相对于本页“不改造”基准计算。</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B2" s="1" t="n"/>
+      <s:c r="C2" s="1" t="n"/>
+      <s:c r="D2" s="1" t="n"/>
+      <s:c r="E2" s="1" t="n"/>
+      <s:c r="F2" s="1" t="n"/>
+    </s:row>
+    <s:row r="4">
+      <s:c r="A4" s="44" t="inlineStr">
+        <s:is>
+          <s:t>项目</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B4" s="44" t="inlineStr">
+        <s:is>
+          <s:t>单位</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C4" s="44" t="inlineStr">
+        <s:is>
+          <s:t>公式/口径</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D4" s="44" t="inlineStr">
+        <s:is>
+          <s:t>计算值</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="E4" s="44" t="inlineStr">
+        <s:is>
+          <s:t>备注</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="F4" s="44" t="inlineStr">
+        <s:is>
+          <s:t>校验</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="5">
+      <s:c r="A5" s="45" t="inlineStr">
+        <s:is>
+          <s:t>灯具数量</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B5" s="45" t="inlineStr">
+        <s:is>
+          <s:t>盏</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C5" s="60" t="inlineStr">
+        <s:is>
+          <s:t>来自Inputs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D5" s="187">
+        <s:f>'02_Inputs'!D6</s:f>
+        <s:v/>
+      </s:c>
+      <s:c r="E5" s="60" t="str"/>
+      <s:c r="F5" s="45" t="inlineStr">
+        <s:is>
+          <s:t>灯杆数量(根)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="G5">
+        <s:f>'02_Inputs'!D49</s:f>
+        <s:v/>
+      </s:c>
+    </s:row>
+    <s:row r="6">
+      <s:c r="A6" s="45" t="inlineStr">
+        <s:is>
+          <s:t>现状单灯功率</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B6" s="45" t="inlineStr">
+        <s:is>
+          <s:t>W/盏</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C6" s="60" t="inlineStr">
+        <s:is>
+          <s:t>来自Inputs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D6" s="187">
+        <s:f>'02_Inputs'!D9</s:f>
+        <s:v/>
+      </s:c>
+      <s:c r="E6" s="60" t="str"/>
+      <s:c r="F6" s="45" t="str"/>
+    </s:row>
+    <s:row r="7">
+      <s:c r="A7" s="45" t="inlineStr">
+        <s:is>
+          <s:t>每日亮灯小时</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B7" s="45" t="inlineStr">
+        <s:is>
+          <s:t>小时/天</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C7" s="60" t="inlineStr">
+        <s:is>
+          <s:t>来自Inputs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D7" s="187">
+        <s:f>'02_Inputs'!D10</s:f>
+        <s:v/>
+      </s:c>
+      <s:c r="E7" s="60" t="str"/>
+      <s:c r="F7" s="45" t="str"/>
+    </s:row>
+    <s:row r="8">
+      <s:c r="A8" s="45" t="inlineStr">
+        <s:is>
+          <s:t>年运行天数</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B8" s="45" t="inlineStr">
+        <s:is>
+          <s:t>天/年</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C8" s="60" t="inlineStr">
+        <s:is>
+          <s:t>来自Inputs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D8" s="187">
+        <s:f>'02_Inputs'!D11</s:f>
+        <s:v/>
+      </s:c>
+      <s:c r="E8" s="60" t="str"/>
+      <s:c r="F8" s="45" t="str"/>
+    </s:row>
+    <s:row r="9">
+      <s:c r="A9" s="45" t="inlineStr">
+        <s:is>
+          <s:t>年运行小时</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B9" s="45" t="inlineStr">
+        <s:is>
+          <s:t>小时/年</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C9" s="60" t="inlineStr">
+        <s:is>
+          <s:t>每日亮灯小时×年运行天数</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D9" s="187">
+        <s:f>D7*D8</s:f>
+        <s:v/>
+      </s:c>
+      <s:c r="E9" s="60" t="str"/>
+      <s:c r="F9" s="45" t="str"/>
+    </s:row>
+    <s:row r="10">
+      <s:c r="A10" s="45" t="inlineStr">
+        <s:is>
+          <s:t>现状年用电量</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B10" s="45" t="inlineStr">
+        <s:is>
+          <s:t>kWh/年</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C10" s="60" t="inlineStr">
+        <s:is>
+          <s:t>灯具数量×单灯功率÷1000×年运行小时</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D10" s="187">
+        <s:f>D5*D6/1000*D9</s:f>
+        <s:v>3073266.0</s:v>
+      </s:c>
+      <s:c r="E10" s="60" t="str"/>
+      <s:c r="F10" s="45" t="str"/>
+    </s:row>
+    <s:row r="11">
+      <s:c r="A11" s="45" t="inlineStr">
+        <s:is>
+          <s:t>电价</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B11" s="45" t="inlineStr">
+        <s:is>
+          <s:t>元/kWh</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C11" s="60" t="inlineStr">
+        <s:is>
+          <s:t>来自Inputs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D11" s="188">
+        <s:f>'02_Inputs'!D8</s:f>
+        <s:v>0.6900001496778997</s:v>
+      </s:c>
+      <s:c r="E11" s="60" t="str"/>
+      <s:c r="F11" s="45" t="str"/>
+    </s:row>
+    <s:row r="12">
+      <s:c r="A12" s="45" t="inlineStr">
+        <s:is>
+          <s:t>基准年电费</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B12" s="45" t="inlineStr">
+        <s:is>
+          <s:t>元/年</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C12" s="60" t="inlineStr">
+        <s:is>
+          <s:t>现状年用电量×电价</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D12" s="189">
+        <s:f>D10*D11</s:f>
+        <s:v>2120554.0</s:v>
+      </s:c>
+      <s:c r="E12" s="60" t="str"/>
+      <s:c r="F12" s="45" t="str"/>
+    </s:row>
+    <s:row r="13">
+      <s:c r="A13" s="45" t="inlineStr">
+        <s:is>
+          <s:t>现状运维单价</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B13" s="45" t="inlineStr">
+        <s:is>
+          <s:t>元/盏/年</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C13" s="60" t="inlineStr">
+        <s:is>
+          <s:t>来自Inputs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D13" s="189">
+        <s:f>'02_Inputs'!D12</s:f>
+        <s:v>133.53699649737302</s:v>
+      </s:c>
+      <s:c r="E13" s="60" t="str"/>
+      <s:c r="F13" s="45" t="str"/>
+    </s:row>
+    <s:row r="14">
+      <s:c r="A14" s="45" t="inlineStr">
+        <s:is>
+          <s:t>基准年运维费</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B14" s="45" t="inlineStr">
+        <s:is>
+          <s:t>元/年</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C14" s="60" t="inlineStr">
+        <s:is>
+          <s:t>灯具数量×现状运维单价</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D14" s="189">
+        <s:f>D5*D13</s:f>
+        <s:v>609997.0</s:v>
+      </s:c>
+      <s:c r="E14" s="60" t="str"/>
+      <s:c r="F14" s="45" t="str"/>
+    </s:row>
+    <s:row r="15">
+      <s:c r="A15" s="79" t="inlineStr">
+        <s:is>
+          <s:t>基准年总成本</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B15" s="79" t="inlineStr">
+        <s:is>
+          <s:t>元/年</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C15" s="89" t="inlineStr">
+        <s:is>
+          <s:t>基准年电费+基准年运维费</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D15" s="190">
+        <s:f>D12+D14</s:f>
+        <s:v>2730551.0</s:v>
+      </s:c>
+      <s:c r="E15" s="89" t="str"/>
+      <s:c r="F15" s="79" t="str"/>
+    </s:row>
+    <s:row r="16">
+      <s:c r="A16" s="79" t="inlineStr">
+        <s:is>
+          <s:t>业主年度服务费预算</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B16" s="79" t="inlineStr">
+        <s:is>
+          <s:t>元/年</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C16" s="89" t="inlineStr">
+        <s:is>
+          <s:t>来自Inputs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D16" s="190">
+        <s:f>'02_Inputs'!D7</s:f>
+        <s:v/>
+      </s:c>
+      <s:c r="E16" s="89" t="str"/>
+      <s:c r="F16" s="79" t="str"/>
+    </s:row>
+    <s:row r="17">
+      <s:c r="A17" s="79" t="inlineStr">
+        <s:is>
+          <s:t>10年业主预算总额</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B17" s="79" t="inlineStr">
+        <s:is>
+          <s:t>元</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C17" s="89" t="inlineStr">
+        <s:is>
+          <s:t>年度预算×模型期</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D17" s="190">
+        <s:f>D16*'02_Inputs'!D5</s:f>
+        <s:v/>
+      </s:c>
+      <s:c r="E17" s="89" t="str"/>
+      <s:c r="F17" s="79" t="str"/>
+    </s:row>
+    <s:row r="18">
+      <s:c r="A18" s="79" t="inlineStr">
+        <s:is>
+          <s:t>10年不改造总成本</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B18" s="79" t="inlineStr">
+        <s:is>
+          <s:t>元</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C18" s="89" t="inlineStr">
+        <s:is>
+          <s:t>年度基准总成本合计，考虑增长率</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D18" s="190">
+        <s:f>SUM('05_Annual_Model'!D8:M8)</s:f>
+        <s:v/>
+      </s:c>
+      <s:c r="E18" s="89" t="str"/>
+      <s:c r="F18" s="79" t="str"/>
+    </s:row>
+  </s:sheetData>
+  <s:mergeCells count="2">
+    <s:mergeCell ref="A2:F2"/>
+    <s:mergeCell ref="A1:F1"/>
+  </s:mergeCells>
+  <s:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</s:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7053,7 +7071,7 @@
       </s:c>
       <s:c r="M24" s="195">
         <s:f>L24+M23</s:f>
-        <s:v>6730600.0</s:v>
+        <s:v>13783630.0</s:v>
       </s:c>
     </s:row>
     <s:row r="25">
@@ -7069,7 +7087,7 @@
       </s:c>
       <s:c r="C25" s="196">
         <s:f>NPV('02_Inputs'!$D$13,D23:M23)+C23</s:f>
-        <s:v>2959712.5361993117</s:v>
+        <s:v>7423046.099119451</s:v>
       </s:c>
       <s:c r="D25" s="193" t="n"/>
       <s:c r="E25" s="193" t="n"/>
@@ -7095,7 +7113,7 @@
       </s:c>
       <s:c r="C26" s="197">
         <s:f>IFERROR(IRR(C23:M23),"n/a")</s:f>
-        <s:v>0.2618003333030041</s:v>
+        <s:v>0.4797080973744201</s:v>
       </s:c>
       <s:c r="D26" s="198" t="n"/>
       <s:c r="E26" s="198" t="n"/>
@@ -7121,7 +7139,7 @@
       </s:c>
       <s:c r="C27" s="199">
         <s:f>IF(C12=0,"n/a",SUM(C23:M23)/C12)</s:f>
-        <s:v>2.901621743798384</s:v>
+        <s:v>4.8943408487314235</s:v>
       </s:c>
       <s:c r="D27" s="198" t="n"/>
       <s:c r="E27" s="198" t="n"/>
@@ -7211,43 +7229,43 @@
       </s:c>
       <s:c r="D31" s="193">
         <s:f>D16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="E31" s="193">
         <s:f>E16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="F31" s="193">
         <s:f>F16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="G31" s="193">
         <s:f>G16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="H31" s="193">
         <s:f>H16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="I31" s="193">
         <s:f>I16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="J31" s="193">
         <s:f>J16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="K31" s="193">
         <s:f>K16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="L31" s="193">
         <s:f>L16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
       <s:c r="M31" s="193">
         <s:f>M16*(1-'04_Mode_Params'!$C$10)</s:f>
-        <s:v>1028000.0</s:v>
+        <s:v>1028003.0</s:v>
       </s:c>
     </s:row>
     <s:row r="32">
@@ -7267,43 +7285,43 @@
       </s:c>
       <s:c r="D32" s="193">
         <s:f>D13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="E32" s="193">
         <s:f>E13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="F32" s="193">
         <s:f>F13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="G32" s="193">
         <s:f>G13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="H32" s="193">
         <s:f>H13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="I32" s="193">
         <s:f>I13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="J32" s="193">
         <s:f>J13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="K32" s="193">
         <s:f>K13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="L32" s="193">
         <s:f>L13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
       <s:c r="M32" s="193">
         <s:f>M13</s:f>
-        <s:v>1637000.0</s:v>
+        <s:v>2342300.0</s:v>
       </s:c>
     </s:row>
     <s:row r="33">
@@ -7379,43 +7397,43 @@
       </s:c>
       <s:c r="D34" s="195">
         <s:f>D31+D32+D33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="E34" s="195">
         <s:f>E31+E32+E33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="F34" s="195">
         <s:f>F31+F32+F33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="G34" s="195">
         <s:f>G31+G32+G33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="H34" s="195">
         <s:f>H31+H32+H33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="I34" s="195">
         <s:f>I31+I32+I33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="J34" s="195">
         <s:f>J31+J32+J33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="K34" s="195">
         <s:f>K31+K32+K33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="L34" s="195">
         <s:f>L31+L32+L33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
       <s:c r="M34" s="195">
         <s:f>M31+M32+M33</s:f>
-        <s:v>2665000.0</s:v>
+        <s:v>3370303.0</s:v>
       </s:c>
     </s:row>
     <s:row r="35">
@@ -7435,43 +7453,43 @@
       </s:c>
       <s:c r="D35" s="195">
         <s:f>D8-D34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="E35" s="195">
         <s:f>E8-E34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="F35" s="195">
         <s:f>F8-F34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="G35" s="195">
         <s:f>G8-G34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="H35" s="195">
         <s:f>H8-H34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="I35" s="195">
         <s:f>I8-I34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="J35" s="195">
         <s:f>J8-J34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="K35" s="195">
         <s:f>K8-K34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="L35" s="195">
         <s:f>L8-L34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
       <s:c r="M35" s="195">
         <s:f>M8-M34</s:f>
-        <s:v>1000.0</s:v>
+        <s:v>-639752.0</s:v>
       </s:c>
     </s:row>
     <s:row r="36">
@@ -7637,43 +7655,43 @@
       </s:c>
       <s:c r="D40" s="193">
         <s:f>MAX(0,('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(1-1))-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="E40" s="193">
         <s:f>MAX(0,('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(2-1))-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="F40" s="193">
         <s:f>MAX(0,('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(3-1))-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="G40" s="193">
         <s:f>MAX(0,('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(4-1))-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="H40" s="193">
         <s:f>MAX(0,('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(5-1))-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="I40" s="193">
         <s:f>MAX(0,('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(6-1))-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="J40" s="193">
         <s:f>MAX(0,MAX((('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(7-1))*0.2),('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(7-1))-'02_Inputs'!$D$46)-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="K40" s="193">
         <s:f>MAX(0,MAX((('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(8-1))*0.2),('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(8-1))-'02_Inputs'!$D$46)-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="L40" s="193">
         <s:f>MAX(0,MAX((('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(9-1))*0.2),('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(9-1))-'02_Inputs'!$D$46)-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="M40" s="193">
         <s:f>MAX(0,MAX((('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(10-1))*0.2),('04_Mode_Params'!$D$6*(1+'02_Inputs'!$D$16)^(10-1))-'02_Inputs'!$D$46)-('02_Inputs'!$D$45/'02_Inputs'!$D$5))</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
     </s:row>
     <s:row r="41">
@@ -8289,7 +8307,7 @@
       </s:c>
       <s:c r="M51" s="195">
         <s:f>L51+M50</s:f>
-        <s:v>15684600.0</s:v>
+        <s:v>16184599.999999976</s:v>
       </s:c>
     </s:row>
     <s:row r="52">
@@ -8305,7 +8323,7 @@
       </s:c>
       <s:c r="C52" s="196">
         <s:f>NPV('02_Inputs'!$D$13,D50:M50)+C50</s:f>
-        <s:v>7907776.500426378</s:v>
+        <s:v>8205507.890886906</s:v>
       </s:c>
       <s:c r="D52" s="193" t="n"/>
       <s:c r="E52" s="193" t="n"/>
@@ -8331,7 +8349,7 @@
       </s:c>
       <s:c r="C53" s="197">
         <s:f>IFERROR(IRR(C50:M50),"n/a")</s:f>
-        <s:v>0.6965192371624709</s:v>
+        <s:v>0.7200751553415916</s:v>
       </s:c>
       <s:c r="D53" s="198" t="n"/>
       <s:c r="E53" s="198" t="n"/>
@@ -8357,7 +8375,7 @@
       </s:c>
       <s:c r="C54" s="199">
         <s:f>IF(C39=0,"n/a",SUM(C50:M50)/C39)</s:f>
-        <s:v>5.431429055772165</s:v>
+        <s:v>5.572695937164491</s:v>
       </s:c>
       <s:c r="D54" s="198" t="n"/>
       <s:c r="E54" s="198" t="n"/>
@@ -8447,43 +8465,43 @@
       </s:c>
       <s:c r="D58" s="193">
         <s:f>D43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="E58" s="193">
         <s:f>E43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="F58" s="193">
         <s:f>F43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="G58" s="193">
         <s:f>G43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="H58" s="193">
         <s:f>H43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="I58" s="193">
         <s:f>I43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="J58" s="193">
         <s:f>J43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="K58" s="193">
         <s:f>K43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="L58" s="193">
         <s:f>L43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
       <s:c r="M58" s="193">
         <s:f>M43*(1-'04_Mode_Params'!$D$10)</s:f>
-        <s:v>411199.9999999999</s:v>
+        <s:v>424110.79999999993</s:v>
       </s:c>
     </s:row>
     <s:row r="59">
@@ -8503,43 +8521,43 @@
       </s:c>
       <s:c r="D59" s="193">
         <s:f>D40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="E59" s="193">
         <s:f>E40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="F59" s="193">
         <s:f>F40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="G59" s="193">
         <s:f>G40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="H59" s="193">
         <s:f>H40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="I59" s="193">
         <s:f>I40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="J59" s="193">
         <s:f>J40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="K59" s="193">
         <s:f>K40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="L59" s="193">
         <s:f>L40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
       <s:c r="M59" s="193">
         <s:f>M40</s:f>
-        <s:v>2250000.0</s:v>
+        <s:v>2300000.0</s:v>
       </s:c>
     </s:row>
     <s:row r="60">
@@ -8615,43 +8633,43 @@
       </s:c>
       <s:c r="D61" s="195">
         <s:f>D58+D59+D60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="E61" s="195">
         <s:f>E58+E59+E60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="F61" s="195">
         <s:f>F58+F59+F60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="G61" s="195">
         <s:f>G58+G59+G60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="H61" s="195">
         <s:f>H58+H59+H60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="I61" s="195">
         <s:f>I58+I59+I60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="J61" s="195">
         <s:f>J58+J59+J60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="K61" s="195">
         <s:f>K58+K59+K60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="L61" s="195">
         <s:f>L58+L59+L60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
       <s:c r="M61" s="195">
         <s:f>M58+M59+M60</s:f>
-        <s:v>2661200.0</s:v>
+        <s:v>2724110.8</s:v>
       </s:c>
     </s:row>
     <s:row r="62">
@@ -8671,43 +8689,43 @@
       </s:c>
       <s:c r="D62" s="195">
         <s:f>D8-D61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="E62" s="195">
         <s:f>E8-E61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="F62" s="195">
         <s:f>F8-F61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="G62" s="195">
         <s:f>G8-G61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="H62" s="195">
         <s:f>H8-H61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="I62" s="195">
         <s:f>I8-I61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="J62" s="195">
         <s:f>J8-J61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="K62" s="195">
         <s:f>K8-K61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="L62" s="195">
         <s:f>L8-L61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
       <s:c r="M62" s="195">
         <s:f>M8-M61</s:f>
-        <s:v>4800.0</s:v>
+        <s:v>6440.200000000186</s:v>
       </s:c>
     </s:row>
     <s:row r="63">
@@ -9232,31 +9250,31 @@
       </s:c>
       <s:c r="B19" s="170">
         <s:f>'03_Baseline'!$D$15-('03_Baseline'!$D$12*(1-0.4)*(1-'04_Mode_Params'!$D$10)+'04_Mode_Params'!$D$6+'02_Inputs'!$D$17)</s:f>
-        <s:v>-817600.0</s:v>
+        <s:v>-841781.3999999999</s:v>
       </s:c>
       <s:c r="C19" s="170">
         <s:f>'03_Baseline'!$D$15-('03_Baseline'!$D$12*(1-0.45)*(1-'04_Mode_Params'!$D$10)+'04_Mode_Params'!$D$6+'02_Inputs'!$D$17)</s:f>
-        <s:v>-714800.0</s:v>
+        <s:v>-735753.7000000002</s:v>
       </s:c>
       <s:c r="D19" s="170">
         <s:f>'03_Baseline'!$D$15-('03_Baseline'!$D$12*(1-0.5)*(1-'04_Mode_Params'!$D$10)+'04_Mode_Params'!$D$6+'02_Inputs'!$D$17)</s:f>
-        <s:v>-612000.0</s:v>
+        <s:v>-597452.0</s:v>
       </s:c>
       <s:c r="E19" s="170">
         <s:f>'03_Baseline'!$D$15-('03_Baseline'!$D$12*(1-0.55)*(1-'04_Mode_Params'!$D$10)+'04_Mode_Params'!$D$6+'02_Inputs'!$D$17)</s:f>
-        <s:v>-509200.0</s:v>
+        <s:v>-523698.2999999998</s:v>
       </s:c>
       <s:c r="F19" s="170">
         <s:f>'03_Baseline'!$D$15-('03_Baseline'!$D$12*(1-0.6)*(1-'04_Mode_Params'!$D$10)+'04_Mode_Params'!$D$6+'02_Inputs'!$D$17)</s:f>
-        <s:v>-406400.0</s:v>
+        <s:v>-417670.6000000001</s:v>
       </s:c>
       <s:c r="G19" s="170">
         <s:f>'03_Baseline'!$D$15-('03_Baseline'!$D$12*(1-0.65)*(1-'04_Mode_Params'!$D$10)+'04_Mode_Params'!$D$6+'02_Inputs'!$D$17)</s:f>
-        <s:v>-303600.0</s:v>
+        <s:v>-311642.8999999999</s:v>
       </s:c>
       <s:c r="H19" s="170">
         <s:f>'03_Baseline'!$D$15-('03_Baseline'!$D$12*(1-0.7)*(1-'04_Mode_Params'!$D$10)+'04_Mode_Params'!$D$6+'02_Inputs'!$D$17)</s:f>
-        <s:v>-200800.0</s:v>
+        <s:v>-205615.2000000002</s:v>
       </s:c>
     </s:row>
     <s:row r="20">

</xml_diff>